<commit_message>
Revise Homework 1 math typesetting and simplify panel task
</commit_message>
<xml_diff>
--- a/assignments/homework-01/MIE446_HW1_NACA2412_Data.xlsx
+++ b/assignments/homework-01/MIE446_HW1_NACA2412_Data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R97d76d8ccb5743bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="Rce3a253223164d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6d78913f12b14aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="Rf41789f0f2af4520"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -496,7 +496,7 @@
       </x:c>
       <x:c r="C6" s="41"/>
       <x:c r="D6" s="13" t="str">
-        <x:v>Use the Data sheet for Question 2. Keep the supplied columns unchanged. Add your own columns for Cp,u, Cp,l, surface slopes, normal and axial integrands, and trapezoidal or panel contributions. Show formulas in the submitted workbook.</x:v>
+        <x:v>Question 2: keep supplied Data unchanged. Compute upper/lower Cp, then normal and axial force contributions for each of 100 panels. Sum the panels and show formulas. No slopes or extra charts.</x:v>
       </x:c>
       <x:c r="E6" s="13"/>
       <x:c r="F6" s="13"/>

</xml_diff>